<commit_message>
Record the scanned board total, not the filtered count, in analytics
The analytics workbook was recording the relevance-filtered count (Product
Design / UI/UX titles only), which read far lower than the number each board
displays — e.g. DOU 76 and Djinni 73 against the 244 and 78 shown on the sites
and in the report's "scanned" totals. That was confusing when compared against
the boards directly.

Record the scanned total instead — the raw count each board returns before the
relevance filter (`scrapers.fetch_all`'s `_totals`): DOU's whole Design category
and Djinni's Product Design + UI/UX tag listing. This mirrors what the sites
report. A source that failed to scrape is absent from `_totals`, so it is stored
as a blank gap rather than a zero, matching the existing convention.

The chart title, module docstring, and README wording are updated to say
"scanned total", and today's seed row is refreshed to 244/78.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/vacancy-analytics.xlsx
+++ b/reports/vacancy-analytics.xlsx
@@ -136,7 +136,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>DOU + Djinni — Product Design / UI/UX вакансії</a:t>
+              <a:t>DOU + Djinni — кількість вакансій на борді</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -617,10 +617,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>76</v>
+        <v>244</v>
       </c>
       <c r="C2" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record the scanned board total, not the filtered count, in analytics (#37)
The analytics workbook was recording the relevance-filtered count (Product
Design / UI/UX titles only), which read far lower than the number each board
displays — e.g. DOU 76 and Djinni 73 against the 244 and 78 shown on the sites
and in the report's "scanned" totals. That was confusing when compared against
the boards directly.

Record the scanned total instead — the raw count each board returns before the
relevance filter (`scrapers.fetch_all`'s `_totals`): DOU's whole Design category
and Djinni's Product Design + UI/UX tag listing. This mirrors what the sites
report. A source that failed to scrape is absent from `_totals`, so it is stored
as a blank gap rather than a zero, matching the existing convention.

The chart title, module docstring, and README wording are updated to say
"scanned total", and today's seed row is refreshed to 244/78.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/vacancy-analytics.xlsx
+++ b/reports/vacancy-analytics.xlsx
@@ -136,7 +136,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>DOU + Djinni — Product Design / UI/UX вакансії</a:t>
+              <a:t>DOU + Djinni — кількість вакансій на борді</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -617,10 +617,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>76</v>
+        <v>244</v>
       </c>
       <c r="C2" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backfill the 2026-09-10 vacancy counts
Adds a data point for 2026-09-10 recovered from the archived report
(reports/report-2026-09-10.md), whose per-source headings show the scanned
totals DOU 254 and Djinni 80 — the same metric the analytics now track. This is
the earliest day with a recoverable scanned total: the 2026-09-08 and 2026-09-09
reports predate the "show scanned totals" change and list only the filtered
count, and nothing exists before 2026-09-08.

The workbook is regenerated from the CSV, so the chart now spans two days.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/vacancy-analytics.xlsx
+++ b/reports/vacancy-analytics.xlsx
@@ -168,12 +168,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2</f>
+              <f>'Counts'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$B$2</f>
+              <f>'Counts'!$B$2:$B$3</f>
             </numRef>
           </val>
         </ser>
@@ -200,12 +200,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2</f>
+              <f>'Counts'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$C$2</f>
+              <f>'Counts'!$C$2:$C$3</f>
             </numRef>
           </val>
         </ser>
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,13 +613,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>254</v>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>244</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>78</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Backfill the 2026-09-10 vacancy counts (#38)
Adds a data point for 2026-09-10 recovered from the archived report
(reports/report-2026-09-10.md), whose per-source headings show the scanned
totals DOU 254 and Djinni 80 — the same metric the analytics now track. This is
the earliest day with a recoverable scanned total: the 2026-09-08 and 2026-09-09
reports predate the "show scanned totals" change and list only the filtered
count, and nothing exists before 2026-09-08.

The workbook is regenerated from the CSV, so the chart now spans two days.

Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/vacancy-analytics.xlsx
+++ b/reports/vacancy-analytics.xlsx
@@ -168,12 +168,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2</f>
+              <f>'Counts'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$B$2</f>
+              <f>'Counts'!$B$2:$B$3</f>
             </numRef>
           </val>
         </ser>
@@ -200,12 +200,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2</f>
+              <f>'Counts'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$C$2</f>
+              <f>'Counts'!$C$2:$C$3</f>
             </numRef>
           </val>
         </ser>
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,13 +613,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>254</v>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>244</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>78</v>
       </c>
     </row>

</xml_diff>